<commit_message>
Actualiza repertorio con materiales del 6 de julio
</commit_message>
<xml_diff>
--- a/data/excel/NaNB V.A.16 (okok).xlsx
+++ b/data/excel/NaNB V.A.16 (okok).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/antonietta/Dropbox/Progetto AISPI FU.HIS.IT./repertorio/testimoni catalogati nel repertorio/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C6D9A757-6D04-D449-A73B-2A33B73BFA0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550D0F2F-8E1C-2F4A-9468-3882CDCC9537}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="25820" windowHeight="16100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="520">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1195" uniqueCount="521">
   <si>
     <t>Íncipit</t>
   </si>
@@ -225,9 +225,6 @@
     </r>
   </si>
   <si>
-    <t>Ningún remedio hay tan bueno / para un duro corazón / como ponelle un bolsón / de doblones en el seno. / Cuando un corazón es duro / más que diamante y acero / ablandarle con dinero / que el dinero ablanda un muro, / que lo más perfecto y bueno / para un duro corazón / es el ponerle un bolsón / de doblones en el seno. / Las damas de nuestros tiempos / tienen ya determinado / de trocar por un ducado / trecientos mil pasatiempos. / De Diana y de Sireno / se ríen y hacen baldón / y lloran por un bolsón / de doblones en el seno. / También ríen del galán / que canta a las doce dadas / con glosas enamoradas / la mañaana de san Juan, / porque no tienen por bueno / el cantar con discricíon / sino tener un bolsón / de doblones en el seno.</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -297,6 +294,140 @@
   </si>
   <si>
     <t>calor tiene, madre</t>
+  </si>
+  <si>
+    <t>22v-23v</t>
+  </si>
+  <si>
+    <t>El pecho se abrasa</t>
+  </si>
+  <si>
+    <t>¡Aire, Dios, y aire / y podrá sufrillo!</t>
+  </si>
+  <si>
+    <t>Haciendo fiestas la corte</t>
+  </si>
+  <si>
+    <t>del gran rey Felipe de Austria</t>
+  </si>
+  <si>
+    <t>23v-26v</t>
+  </si>
+  <si>
+    <t>Riñó con Juanilla</t>
+  </si>
+  <si>
+    <t>su hermana Miguela</t>
+  </si>
+  <si>
+    <t>26v-28v</t>
+  </si>
+  <si>
+    <t>Letra</t>
+  </si>
+  <si>
+    <t>polimetría</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>s</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>í</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>Eres ni</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ñ</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t>a y has amor</t>
+    </r>
+  </si>
+  <si>
+    <t>alférez mayor del reino</t>
+  </si>
+  <si>
+    <t>29r-32r</t>
+  </si>
+  <si>
+    <t>Otro</t>
+  </si>
+  <si>
+    <t>Si de amor te dicen</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>que es</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> dulce manjar</t>
+    </r>
+  </si>
+  <si>
+    <t>32v-33v</t>
+  </si>
+  <si>
+    <t>Aunque tus amigos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¡No le comas, niña / que es como rejalgar! </t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Doña Blanca está en Sidonia</t>
+    </r>
+  </si>
+  <si>
+    <t>contando su historia amarga</t>
   </si>
   <si>
     <r>
@@ -305,7 +436,7 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t>y podr</t>
+      <t>¿qué mal habr</t>
     </r>
     <r>
       <rPr>
@@ -322,123 +453,118 @@
         <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
       </rPr>
-      <t xml:space="preserve"> sufrillo!</t>
-    </r>
-  </si>
-  <si>
-    <t>22v-23v</t>
-  </si>
-  <si>
-    <t>El pecho se abrasa</t>
-  </si>
-  <si>
-    <t>¡Aire, Dios, y aire / y podrá sufrillo!</t>
-  </si>
-  <si>
-    <t>Haciendo fiestas la corte</t>
-  </si>
-  <si>
-    <t>del gran rey Felipe de Austria</t>
-  </si>
-  <si>
-    <t>23v-26v</t>
-  </si>
-  <si>
-    <t>Riñó con Juanilla</t>
-  </si>
-  <si>
-    <t>su hermana Miguela</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>¿qué har</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+      <t xml:space="preserve"> que no haga?</t>
+    </r>
+  </si>
+  <si>
+    <t>33v-34r</t>
+  </si>
+  <si>
+    <t>Carillo, a risa provoca</t>
+  </si>
+  <si>
+    <t>34v-35r</t>
+  </si>
+  <si>
+    <t>Entrando una tarde a vella</t>
+  </si>
+  <si>
+    <t>Tiniendo de vos tal prenda</t>
+  </si>
+  <si>
+    <t>no hay prenda que a mí me prenda</t>
+  </si>
+  <si>
+    <t>Zarabanda</t>
+  </si>
+  <si>
+    <t>estribote</t>
+  </si>
+  <si>
+    <t>La prenda que me dejastes</t>
+  </si>
+  <si>
+    <t>Tiniendo de vos tal prenda, / no hay prenda que a mí me prenda.</t>
+  </si>
+  <si>
+    <t>Alegre porque moría</t>
+  </si>
+  <si>
+    <t>36v-37v</t>
+  </si>
+  <si>
+    <t>[Liñán de Riaza, Pedro]</t>
+  </si>
+  <si>
+    <t>malo me siento.</t>
+  </si>
+  <si>
+    <t>No sigas a Silvia, Bras</t>
+  </si>
+  <si>
+    <t>por verte favorecer</t>
+  </si>
+  <si>
+    <t>37v-38v</t>
+  </si>
+  <si>
+    <t>Otra letrilla</t>
+  </si>
+  <si>
+    <t xml:space="preserve">villancico </t>
+  </si>
+  <si>
+    <t>Si no tienes qué le dar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">siendo amiga de Tomás? </t>
+  </si>
+  <si>
+    <t>La más bella niña</t>
+  </si>
+  <si>
+    <t>de nuestro lugar</t>
+  </si>
+  <si>
+    <t>39r-40r</t>
+  </si>
+  <si>
+    <t>Romance contrahecho</t>
+  </si>
+  <si>
+    <t>¡Dejadme llorar, / orillas de la mar!</t>
+  </si>
+  <si>
+    <t>fortuna de su tesoro</t>
+  </si>
+  <si>
+    <t>40r-41r</t>
+  </si>
+  <si>
+    <t>Que haya fortuna tratado</t>
+  </si>
+  <si>
+    <t>y a mí que me tome el toro.</t>
+  </si>
+  <si>
+    <t>Noble desengaño,</t>
+  </si>
+  <si>
+    <t>gracias doy al cielo</t>
+  </si>
+  <si>
+    <t>41r-44v</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>ás quando mayor?</t>
-    </r>
-  </si>
-  <si>
-    <t>26v-28v</t>
-  </si>
-  <si>
-    <t>Letra</t>
-  </si>
-  <si>
-    <t>polimetría</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>s</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>í</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>Eres ni</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>ñ</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>a y has amor</t>
-    </r>
-  </si>
-  <si>
-    <t>Aquel rayo de la guerra</t>
-  </si>
-  <si>
-    <t>alférez mayor del reino</t>
-  </si>
-  <si>
-    <t>29r-32r</t>
-  </si>
-  <si>
-    <t>Otro</t>
-  </si>
-  <si>
-    <t>Si de amor te dicen</t>
-  </si>
-  <si>
+      <t xml:space="preserve">Bien haya </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -446,7 +572,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>que es</t>
+      <t>aquel</t>
     </r>
     <r>
       <rPr>
@@ -455,20 +581,38 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> dulce manjar</t>
-    </r>
-  </si>
-  <si>
-    <t>que es como rejalgar!</t>
-  </si>
-  <si>
-    <t>32v-33v</t>
-  </si>
-  <si>
-    <t>Aunque tus amigos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">¡No le comas, niña / que es como rejalgar! </t>
+      <t xml:space="preserve"> que no cura</t>
+    </r>
+  </si>
+  <si>
+    <t>de melindres ni locura</t>
+  </si>
+  <si>
+    <t>44v-48v</t>
+  </si>
+  <si>
+    <t>Ensaladilla</t>
+  </si>
+  <si>
+    <t>Quien tratare a ley de Coria</t>
+  </si>
+  <si>
+    <t>A ti, Venus, invoco solamente</t>
+  </si>
+  <si>
+    <t>no curo de Aganipe ni Ipocrene</t>
+  </si>
+  <si>
+    <t>49r-54r</t>
+  </si>
+  <si>
+    <t>Cuento de un pintor</t>
+  </si>
+  <si>
+    <t>tercetos encadenados</t>
+  </si>
+  <si>
+    <t>Galanes y caballeros</t>
   </si>
   <si>
     <r>
@@ -478,149 +622,61 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>Doña Blanca está en Sidonia</t>
-    </r>
-  </si>
-  <si>
-    <t>contando su historia amarga</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t>¿qué mal habr</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
+      <t>que de Amor seguís el bando</t>
+    </r>
+  </si>
+  <si>
+    <t>54v-56r</t>
+  </si>
+  <si>
+    <t>[Padilla, Pedro de]</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>á</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Aptos Narrow"/>
-      </rPr>
-      <t xml:space="preserve"> que no haga?</t>
-    </r>
-  </si>
-  <si>
-    <t>33v-34r</t>
-  </si>
-  <si>
-    <t>Carillo, a risa provoca</t>
-  </si>
-  <si>
-    <t>una nueva maravilla:</t>
-  </si>
-  <si>
-    <t>34v-35r</t>
-  </si>
-  <si>
-    <t>Entrando una tarde a vella</t>
-  </si>
-  <si>
-    <t>Tiniendo de vos tal prenda</t>
-  </si>
-  <si>
-    <t>no hay prenda que a mí me prenda</t>
-  </si>
-  <si>
-    <t>Zarabanda</t>
-  </si>
-  <si>
-    <t>estribote</t>
-  </si>
-  <si>
-    <t>La prenda que me dejastes</t>
-  </si>
-  <si>
-    <t>Tiniendo de vos tal prenda, / no hay prenda que a mí me prenda.</t>
-  </si>
-  <si>
-    <t>Alegre porque moría</t>
-  </si>
-  <si>
-    <t>en la fee de su tormento</t>
-  </si>
-  <si>
-    <t>36v-37v</t>
-  </si>
-  <si>
-    <t>[Liñán de Riaza, Pedro]</t>
-  </si>
-  <si>
-    <t>malo me siento.</t>
-  </si>
-  <si>
-    <t>No sigas a Silvia, Bras</t>
-  </si>
-  <si>
-    <t>por verte favorecer</t>
-  </si>
-  <si>
-    <t>37v-38v</t>
-  </si>
-  <si>
-    <t>Otra letrilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">villancico </t>
-  </si>
-  <si>
-    <t>Si no tienes qué le dar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">siendo amiga de Tomás? </t>
-  </si>
-  <si>
-    <t>La más bella niña</t>
-  </si>
-  <si>
-    <t>de nuestro lugar</t>
-  </si>
-  <si>
-    <t>orillas de la mar!</t>
-  </si>
-  <si>
-    <t>39r-40r</t>
-  </si>
-  <si>
-    <t>Romance contrahecho</t>
-  </si>
-  <si>
-    <t>¡Dejadme llorar, / orillas de la mar!</t>
-  </si>
-  <si>
-    <t>Que con quatro mil reparta</t>
-  </si>
-  <si>
-    <t>fortuna de su tesoro</t>
-  </si>
-  <si>
-    <t>40r-41r</t>
-  </si>
-  <si>
-    <t>Que haya fortuna tratado</t>
-  </si>
-  <si>
-    <t>y a mí que me tome el toro.</t>
-  </si>
-  <si>
-    <t>Noble desengaño,</t>
-  </si>
-  <si>
-    <t>gracias doy al cielo</t>
-  </si>
-  <si>
-    <t>41r-44v</t>
+      <t>¿Quién quiere un mozo galán y dispuesto</t>
+    </r>
+  </si>
+  <si>
+    <t>56v-57v</t>
+  </si>
+  <si>
+    <t>y tiene mil gracias aliende de aquesto.</t>
+  </si>
+  <si>
+    <t>Si las damas de la Corte</t>
+  </si>
+  <si>
+    <t>quieren, por dar una mano</t>
+  </si>
+  <si>
+    <t>58rv</t>
+  </si>
+  <si>
+    <t>que yo soy nacido en el Potro.</t>
+  </si>
+  <si>
+    <t>Bella pastorcica</t>
+  </si>
+  <si>
+    <t>de la tez morena</t>
+  </si>
+  <si>
+    <t>59rv</t>
+  </si>
+  <si>
+    <t>Pastorcica hermosa,</t>
+  </si>
+  <si>
+    <t>No miente quien dice / que me das pena.</t>
+  </si>
+  <si>
+    <t>Al camino de Toledo</t>
   </si>
   <si>
     <r>
@@ -630,8 +686,19 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">Bien haya </t>
-    </r>
+      <t>adonde dejó empeñada</t>
+    </r>
+  </si>
+  <si>
+    <t>60r-61v</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Romance </t>
+  </si>
+  <si>
+    <t>Que ausencia sin mudanza / comienza en celos y en morir acaba.</t>
+  </si>
+  <si>
     <r>
       <rPr>
         <sz val="11"/>
@@ -639,7 +706,7 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>aquel</t>
+      <t>Ahora,</t>
     </r>
     <r>
       <rPr>
@@ -648,40 +715,8 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve"> que no cura</t>
-    </r>
-  </si>
-  <si>
-    <t>de melindres ni locura</t>
-  </si>
-  <si>
-    <t>44v-48v</t>
-  </si>
-  <si>
-    <t>Ensaladilla</t>
-  </si>
-  <si>
-    <t>Quien tratare a ley de Coria</t>
-  </si>
-  <si>
-    <t>A ti, Venus, invoco solamente</t>
-  </si>
-  <si>
-    <t>no curo de Aganipe ni Ipocrene</t>
-  </si>
-  <si>
-    <t>49r-54r</t>
-  </si>
-  <si>
-    <t>Cuento de un pintor</t>
-  </si>
-  <si>
-    <t>tercetos encadenados</t>
-  </si>
-  <si>
-    <t>Galanes y caballeros</t>
-  </si>
-  <si>
+      <t xml:space="preserve"> Tirsi, </t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -689,16 +724,8 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>que de Amor seguís el bando</t>
-    </r>
-  </si>
-  <si>
-    <t>54v-56r</t>
-  </si>
-  <si>
-    <t>[Padilla, Pedro de]</t>
-  </si>
-  <si>
+      <t>que el</t>
+    </r>
     <r>
       <rPr>
         <sz val="11"/>
@@ -706,50 +733,17 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>¿Quién quiere un mozo galán y dispuesto</t>
-    </r>
-  </si>
-  <si>
-    <t>que tañe y que danza y tira a la barra</t>
-  </si>
-  <si>
-    <t>56v-57v</t>
-  </si>
-  <si>
-    <t>y tiene mil gracias aliende de aquesto.</t>
-  </si>
-  <si>
-    <t>Si las damas de la Corte</t>
-  </si>
-  <si>
-    <t>quieren, por dar una mano</t>
-  </si>
-  <si>
-    <t>58rv</t>
-  </si>
-  <si>
-    <t>que yo soy nacido en el Potro.</t>
-  </si>
-  <si>
-    <t>Bella pastorcica</t>
-  </si>
-  <si>
-    <t>de la tez morena</t>
-  </si>
-  <si>
-    <t>59rv</t>
-  </si>
-  <si>
-    <t>Pastorcica hermosa,</t>
-  </si>
-  <si>
-    <t>No miente quien dice / que me das pena.</t>
-  </si>
-  <si>
-    <t>Bella pastorcica, / de la tez morena, / no miente quien dice / que me das pena. / Pastorcica hermosa / que gozáis sigura / de nueva hermosura / la palma dichosa. / beldad milagrosa / que el alma encadena, / no miente quien dice / que me das pena. / Dicen que miré / a unos ojos claros / y que es deuda amaros; / el alma que os ve / presa la dejé / en vuestra cadena. / No miente quien dice / que me das pena.</t>
-  </si>
-  <si>
-    <t>Al camino de Toledo</t>
+      <t xml:space="preserve"> tiempo</t>
+    </r>
+  </si>
+  <si>
+    <t>toma residencia al alma</t>
+  </si>
+  <si>
+    <t>[vanamente creída y adorada!]</t>
+  </si>
+  <si>
+    <t>62rv</t>
   </si>
   <si>
     <r>
@@ -759,73 +753,6 @@
         <rFont val="Calibri"/>
         <family val="2"/>
       </rPr>
-      <t>adonde dejó empeñada</t>
-    </r>
-  </si>
-  <si>
-    <t>60r-61v</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Romance </t>
-  </si>
-  <si>
-    <t>Que ausencia sin mudanza / comienza en celos y en morir acaba.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Ahora,</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Tirsi, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>que el</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> tiempo</t>
-    </r>
-  </si>
-  <si>
-    <t>toma residencia al alma</t>
-  </si>
-  <si>
-    <t>[vanamente creída y adorada!]</t>
-  </si>
-  <si>
-    <t>62rv</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
       <t>¡Oh, Edad falsa, / vanamente creída y adorada!</t>
     </r>
   </si>
@@ -842,9 +769,6 @@
     <t xml:space="preserve">Decenas </t>
   </si>
   <si>
-    <t>[Argensola, Lupercio Leonardo ]</t>
-  </si>
-  <si>
     <t>Niña, acuérdate de mí</t>
   </si>
   <si>
@@ -863,9 +787,6 @@
     <t>de la boca de Medoro</t>
   </si>
   <si>
-    <t xml:space="preserve">invidioso, invidioso! </t>
-  </si>
-  <si>
     <t>65v-66v</t>
   </si>
   <si>
@@ -875,50 +796,9 @@
     <t xml:space="preserve">¡Oh, moro venturoso / que a todo el mundo tienes / invidioso, invidioso! </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>«</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>¡Arriba!</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">» </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>gritaban todos</t>
-    </r>
-  </si>
-  <si>
     <t>los que dan asalto a Baza</t>
   </si>
   <si>
-    <t>arriba, arriba, arriba!</t>
-  </si>
-  <si>
     <t>67r-68r</t>
   </si>
   <si>
@@ -943,26 +823,6 @@
     <t xml:space="preserve">Si fias en mis amores </t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>«</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>Muerte, si te das tal prisa</t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">en llevarme a mi Zerbino </t>
   </si>
   <si>
@@ -975,26 +835,6 @@
     <t xml:space="preserve"> Zamudio, Catalina</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t>«</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Junto a esta laguna </t>
-    </r>
-  </si>
-  <si>
     <t xml:space="preserve">cuyo seno grande </t>
   </si>
   <si>
@@ -1172,9 +1012,6 @@
     <t>97v-99r</t>
   </si>
   <si>
-    <t>Púsoseme el sol</t>
-  </si>
-  <si>
     <t>saliome la luna</t>
   </si>
   <si>
@@ -1238,9 +1075,6 @@
     <t>¡Alarga, morenica, el paso / que me canso!</t>
   </si>
   <si>
-    <t>¡Dura, pensamiento</t>
-  </si>
-  <si>
     <t>que me das contento!</t>
   </si>
   <si>
@@ -1286,27 +1120,18 @@
     <t>110v-111r</t>
   </si>
   <si>
-    <t>A la vista de Tarifa</t>
-  </si>
-  <si>
     <t>poco más de media legua</t>
   </si>
   <si>
     <t>111v-112v</t>
   </si>
   <si>
-    <t>Rogáselo, madre</t>
-  </si>
-  <si>
     <t>rogáselo al niño</t>
   </si>
   <si>
     <t>113r-115r</t>
   </si>
   <si>
-    <t>Ay, memoria amarga</t>
-  </si>
-  <si>
     <t>dulce tesorera</t>
   </si>
   <si>
@@ -1353,9 +1178,6 @@
   </si>
   <si>
     <t>Romance a una mujer de un escribano</t>
-  </si>
-  <si>
-    <t>El que más amaba, madre</t>
   </si>
   <si>
     <t>se me fue</t>
@@ -2919,13 +2741,272 @@
   </si>
   <si>
     <t>huérfana, moza y sola.</t>
+  </si>
+  <si>
+    <t>[Leonardo Argensola, Lupercio]</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Ningún remedio hay tan bueno / para un duro corazón / como ponelle un bolsón / de doblones en el seno</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. / Cuando un corazón es duro / más que diamante y acero / ablandarle con dinero / que el dinero ablanda un muro, / que lo más perfecto y bueno / para un duro corazón / es el ponerle un bolsón / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>de doblones en el seno</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. / Las damas de nuestros tiempos / tienen ya determinado / de trocar por un ducado / trecientos mil pasatiempos. / De Diana y de Sireno / se ríen y hacen baldón / y lloran por un bolsón / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>de doblones en el seno</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. / También ríen del galán / que canta a las doce dadas / con glosas enamoradas / la mañana de san Juan, / porque no tienen por bueno / el cantar con discrecíon / sino tener un bolsón / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>de doblones en el seno</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>Bella pastorcica, / de la tez morena, / no miente quien dice / que me das pena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. / Pastorcica hermosa / que gozáis sigura / de nueva hermosura / la palma dichosa. / Beldad milagrosa / que el alma encadena, / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>no miente quien dice / que me das pena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">. / Dicen que miré / a unos ojos claros / y que es deuda amaros; / el alma que os ve / presa la dejé / en vuestra cadena. / </t>
+    </r>
+    <r>
+      <rPr>
+        <i/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>No miente quien dice / que me das pena</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>¿qué har</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>ás cuando mayor?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>y podr</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>á</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+      </rPr>
+      <t xml:space="preserve"> sufrillo.</t>
+    </r>
+  </si>
+  <si>
+    <t>Aquel rayo de la guerra,</t>
+  </si>
+  <si>
+    <t>que es como rejalgar.</t>
+  </si>
+  <si>
+    <t>una nueva maravilla</t>
+  </si>
+  <si>
+    <t>en la fe de su tormento</t>
+  </si>
+  <si>
+    <t>orillas de la mar.</t>
+  </si>
+  <si>
+    <t>Que con cuatro mil reparta</t>
+  </si>
+  <si>
+    <t>que tañe y que danza y tira a la barra?</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>"¡Arriba!"</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>gritaban todos</t>
+    </r>
+  </si>
+  <si>
+    <t>Muerte, si te das tal prisa</t>
+  </si>
+  <si>
+    <t>¡arriba, arriba, arriba!</t>
+  </si>
+  <si>
+    <t xml:space="preserve">¡invidioso, invidioso! </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Junto a esta laguna </t>
+  </si>
+  <si>
+    <t>Púsoseme el sol,</t>
+  </si>
+  <si>
+    <t>¡Dura, pensamiento,</t>
+  </si>
+  <si>
+    <t>Madre, la mi madre,</t>
+  </si>
+  <si>
+    <t>A la vista de Tarifa,</t>
+  </si>
+  <si>
+    <t>Rogáselo, madre,</t>
+  </si>
+  <si>
+    <t>Ay, memoria amarga,</t>
+  </si>
+  <si>
+    <t>El que más amaba, madre,</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -3054,6 +3135,13 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -3516,13 +3604,13 @@
         <v>15</v>
       </c>
       <c r="Q1" s="8" t="s">
-        <v>512</v>
+        <v>489</v>
       </c>
       <c r="R1" s="9" t="s">
-        <v>514</v>
+        <v>491</v>
       </c>
       <c r="S1" s="9" t="s">
-        <v>513</v>
+        <v>490</v>
       </c>
     </row>
     <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3533,7 +3621,7 @@
         <v>17</v>
       </c>
       <c r="C2" s="11" t="s">
-        <v>501</v>
+        <v>478</v>
       </c>
       <c r="D2" s="12" t="s">
         <v>18</v>
@@ -3548,13 +3636,13 @@
         <v>20</v>
       </c>
       <c r="H2" s="10" t="s">
-        <v>364</v>
+        <v>341</v>
       </c>
       <c r="I2" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J2" s="13" t="s">
-        <v>368</v>
+        <v>345</v>
       </c>
       <c r="K2" s="11" t="s">
         <v>22</v>
@@ -3588,7 +3676,7 @@
         <v>26</v>
       </c>
       <c r="C3" s="11" t="s">
-        <v>502</v>
+        <v>479</v>
       </c>
       <c r="D3" s="12" t="s">
         <v>18</v>
@@ -3609,7 +3697,7 @@
         <v>21</v>
       </c>
       <c r="J3" s="13" t="s">
-        <v>369</v>
+        <v>346</v>
       </c>
       <c r="K3" s="11" t="s">
         <v>22</v>
@@ -3643,7 +3731,7 @@
         <v>31</v>
       </c>
       <c r="C4" s="11" t="s">
-        <v>503</v>
+        <v>480</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>18</v>
@@ -3664,7 +3752,7 @@
         <v>34</v>
       </c>
       <c r="J4" s="13" t="s">
-        <v>370</v>
+        <v>347</v>
       </c>
       <c r="K4" s="11" t="s">
         <v>22</v>
@@ -3698,7 +3786,7 @@
         <v>36</v>
       </c>
       <c r="C5" s="11" t="s">
-        <v>504</v>
+        <v>481</v>
       </c>
       <c r="D5" s="12" t="s">
         <v>18</v>
@@ -3719,7 +3807,7 @@
         <v>21</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>371</v>
+        <v>348</v>
       </c>
       <c r="K5" s="11" t="s">
         <v>22</v>
@@ -3753,7 +3841,7 @@
         <v>40</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>505</v>
+        <v>482</v>
       </c>
       <c r="D6" s="12" t="s">
         <v>18</v>
@@ -3774,7 +3862,7 @@
         <v>21</v>
       </c>
       <c r="J6" s="13" t="s">
-        <v>372</v>
+        <v>349</v>
       </c>
       <c r="K6" s="11" t="s">
         <v>22</v>
@@ -3808,7 +3896,7 @@
         <v>44</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>506</v>
+        <v>483</v>
       </c>
       <c r="D7" s="12" t="s">
         <v>18</v>
@@ -3829,7 +3917,7 @@
         <v>58</v>
       </c>
       <c r="J7" s="37" t="s">
-        <v>374</v>
+        <v>351</v>
       </c>
       <c r="K7" s="11" t="s">
         <v>48</v>
@@ -3847,7 +3935,7 @@
         <v>48</v>
       </c>
       <c r="P7" s="14" t="s">
-        <v>433</v>
+        <v>410</v>
       </c>
       <c r="Q7" s="10" t="s">
         <v>24</v>
@@ -3863,7 +3951,7 @@
         <v>51</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>507</v>
+        <v>484</v>
       </c>
       <c r="D8" s="12" t="s">
         <v>18</v>
@@ -3884,7 +3972,7 @@
         <v>21</v>
       </c>
       <c r="J8" s="16" t="s">
-        <v>373</v>
+        <v>350</v>
       </c>
       <c r="K8" s="17" t="s">
         <v>22</v>
@@ -3918,7 +4006,7 @@
         <v>55</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="D9" s="12" t="s">
         <v>18</v>
@@ -3939,7 +4027,7 @@
         <v>58</v>
       </c>
       <c r="J9" s="37" t="s">
-        <v>374</v>
+        <v>351</v>
       </c>
       <c r="K9" s="17" t="s">
         <v>48</v>
@@ -3957,27 +4045,27 @@
         <v>48</v>
       </c>
       <c r="P9" s="14" t="s">
-        <v>434</v>
+        <v>411</v>
       </c>
       <c r="Q9" s="10" t="s">
         <v>53</v>
       </c>
       <c r="R9" s="12" t="s">
-        <v>60</v>
+        <v>498</v>
       </c>
       <c r="S9" s="33" t="s">
-        <v>363</v>
+        <v>340</v>
       </c>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="10" t="s">
+        <v>60</v>
+      </c>
+      <c r="B10" s="10" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>62</v>
-      </c>
       <c r="C10" s="15" t="s">
-        <v>508</v>
+        <v>485</v>
       </c>
       <c r="D10" s="12" t="s">
         <v>18</v>
@@ -3986,10 +4074,10 @@
         <v>9</v>
       </c>
       <c r="F10" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="G10" s="10" t="s">
         <v>63</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>64</v>
       </c>
       <c r="H10" s="14" t="s">
         <v>42</v>
@@ -3998,7 +4086,7 @@
         <v>58</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>429</v>
+        <v>406</v>
       </c>
       <c r="K10" s="17" t="s">
         <v>22</v>
@@ -4026,13 +4114,13 @@
     </row>
     <row r="11" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>65</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>66</v>
-      </c>
       <c r="C11" s="15" t="s">
-        <v>509</v>
+        <v>486</v>
       </c>
       <c r="D11" s="12" t="s">
         <v>18</v>
@@ -4041,7 +4129,7 @@
         <v>10</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="G11" s="10" t="s">
         <v>46</v>
@@ -4053,13 +4141,13 @@
         <v>47</v>
       </c>
       <c r="J11" s="36" t="s">
-        <v>375</v>
+        <v>352</v>
       </c>
       <c r="K11" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L11" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="M11" s="11" t="s">
         <v>22</v>
@@ -4071,7 +4159,7 @@
         <v>48</v>
       </c>
       <c r="P11" s="14" t="s">
-        <v>435</v>
+        <v>412</v>
       </c>
       <c r="Q11" s="10" t="s">
         <v>53</v>
@@ -4081,13 +4169,13 @@
     </row>
     <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B12" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>70</v>
-      </c>
       <c r="C12" s="15" t="s">
-        <v>510</v>
+        <v>487</v>
       </c>
       <c r="D12" s="12" t="s">
         <v>18</v>
@@ -4096,7 +4184,7 @@
         <v>11</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="G12" s="10" t="s">
         <v>33</v>
@@ -4108,7 +4196,7 @@
         <v>21</v>
       </c>
       <c r="J12" s="16" t="s">
-        <v>376</v>
+        <v>353</v>
       </c>
       <c r="K12" s="17" t="s">
         <v>22</v>
@@ -4126,7 +4214,7 @@
         <v>48</v>
       </c>
       <c r="P12" s="14" t="s">
-        <v>436</v>
+        <v>413</v>
       </c>
       <c r="Q12" s="10" t="s">
         <v>53</v>
@@ -4136,13 +4224,13 @@
     </row>
     <row r="13" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="14" t="s">
+        <v>71</v>
+      </c>
+      <c r="B13" s="14" t="s">
         <v>72</v>
       </c>
-      <c r="B13" s="14" t="s">
-        <v>73</v>
-      </c>
       <c r="C13" s="15" t="s">
-        <v>74</v>
+        <v>501</v>
       </c>
       <c r="D13" s="12" t="s">
         <v>18</v>
@@ -4151,7 +4239,7 @@
         <v>12</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="G13" s="10" t="s">
         <v>46</v>
@@ -4163,13 +4251,13 @@
         <v>58</v>
       </c>
       <c r="J13" s="37" t="s">
-        <v>377</v>
+        <v>354</v>
       </c>
       <c r="K13" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L13" s="10" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="M13" s="11" t="s">
         <v>22</v>
@@ -4181,7 +4269,7 @@
         <v>48</v>
       </c>
       <c r="P13" s="14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="Q13" s="10" t="s">
         <v>53</v>
@@ -4191,13 +4279,13 @@
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="10" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="B14" s="14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>500</v>
+        <v>477</v>
       </c>
       <c r="D14" s="12" t="s">
         <v>18</v>
@@ -4206,7 +4294,7 @@
         <v>13</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>38</v>
@@ -4218,7 +4306,7 @@
         <v>21</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="K14" s="17" t="s">
         <v>22</v>
@@ -4246,13 +4334,13 @@
     </row>
     <row r="15" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="14" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>83</v>
+        <v>500</v>
       </c>
       <c r="D15" s="12" t="s">
         <v>18</v>
@@ -4261,19 +4349,19 @@
         <v>14</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H15" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>431</v>
+        <v>408</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>379</v>
+        <v>356</v>
       </c>
       <c r="K15" s="17" t="s">
         <v>22</v>
@@ -4282,16 +4370,16 @@
         <v>23</v>
       </c>
       <c r="M15" s="11" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="N15" s="11" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="O15" s="18" t="s">
         <v>48</v>
       </c>
       <c r="P15" s="41" t="s">
-        <v>515</v>
+        <v>492</v>
       </c>
       <c r="Q15" s="10" t="s">
         <v>53</v>
@@ -4301,13 +4389,13 @@
     </row>
     <row r="16" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="10" t="s">
-        <v>89</v>
+        <v>502</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>499</v>
+        <v>476</v>
       </c>
       <c r="D16" s="12" t="s">
         <v>18</v>
@@ -4316,10 +4404,10 @@
         <v>15</v>
       </c>
       <c r="F16" s="10" t="s">
-        <v>91</v>
+        <v>87</v>
       </c>
       <c r="G16" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H16" s="14" t="s">
         <v>42</v>
@@ -4328,7 +4416,7 @@
         <v>21</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>378</v>
+        <v>355</v>
       </c>
       <c r="K16" s="17" t="s">
         <v>22</v>
@@ -4356,13 +4444,13 @@
     </row>
     <row r="17" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="14" t="s">
-        <v>93</v>
+        <v>89</v>
       </c>
       <c r="B17" s="14" t="s">
-        <v>94</v>
+        <v>90</v>
       </c>
       <c r="C17" s="15" t="s">
-        <v>95</v>
+        <v>503</v>
       </c>
       <c r="D17" s="12" t="s">
         <v>18</v>
@@ -4371,10 +4459,10 @@
         <v>16</v>
       </c>
       <c r="F17" s="10" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="G17" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H17" s="10" t="s">
         <v>29</v>
@@ -4383,13 +4471,13 @@
         <v>47</v>
       </c>
       <c r="J17" s="36" t="s">
-        <v>380</v>
+        <v>357</v>
       </c>
       <c r="K17" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L17" s="10" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="M17" s="11" t="s">
         <v>22</v>
@@ -4401,7 +4489,7 @@
         <v>48</v>
       </c>
       <c r="P17" s="14" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="Q17" s="10" t="s">
         <v>53</v>
@@ -4411,13 +4499,13 @@
     </row>
     <row r="18" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="10" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B18" s="10" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="C18" s="15" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="D18" s="12" t="s">
         <v>18</v>
@@ -4426,7 +4514,7 @@
         <v>17</v>
       </c>
       <c r="F18" s="10" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="G18" s="10" t="s">
         <v>38</v>
@@ -4438,7 +4526,7 @@
         <v>21</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>381</v>
+        <v>358</v>
       </c>
       <c r="K18" s="17" t="s">
         <v>22</v>
@@ -4466,13 +4554,13 @@
     </row>
     <row r="19" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="14" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>104</v>
+        <v>504</v>
       </c>
       <c r="C19" s="15" t="s">
-        <v>498</v>
+        <v>475</v>
       </c>
       <c r="D19" s="12" t="s">
         <v>18</v>
@@ -4481,10 +4569,10 @@
         <v>18</v>
       </c>
       <c r="F19" s="14" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="G19" s="14" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H19" s="10" t="s">
         <v>29</v>
@@ -4493,13 +4581,13 @@
         <v>58</v>
       </c>
       <c r="J19" s="37" t="s">
-        <v>374</v>
+        <v>351</v>
       </c>
       <c r="K19" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L19" s="10" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="M19" s="11" t="s">
         <v>22</v>
@@ -4511,7 +4599,7 @@
         <v>48</v>
       </c>
       <c r="P19" s="14" t="s">
-        <v>437</v>
+        <v>414</v>
       </c>
       <c r="Q19" s="10" t="s">
         <v>53</v>
@@ -4521,13 +4609,13 @@
     </row>
     <row r="20" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14" t="s">
-        <v>107</v>
+        <v>101</v>
       </c>
       <c r="B20" s="14" t="s">
-        <v>108</v>
+        <v>102</v>
       </c>
       <c r="C20" s="15" t="s">
-        <v>497</v>
+        <v>474</v>
       </c>
       <c r="D20" s="12" t="s">
         <v>18</v>
@@ -4536,25 +4624,25 @@
         <v>19</v>
       </c>
       <c r="F20" s="10" t="s">
-        <v>511</v>
+        <v>488</v>
       </c>
       <c r="G20" s="10" t="s">
-        <v>109</v>
+        <v>103</v>
       </c>
       <c r="H20" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I20" s="14" t="s">
-        <v>110</v>
+        <v>104</v>
       </c>
       <c r="J20" s="23" t="s">
-        <v>382</v>
+        <v>359</v>
       </c>
       <c r="K20" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L20" s="10" t="s">
-        <v>111</v>
+        <v>105</v>
       </c>
       <c r="M20" s="11" t="s">
         <v>22</v>
@@ -4566,7 +4654,7 @@
         <v>48</v>
       </c>
       <c r="P20" s="14" t="s">
-        <v>112</v>
+        <v>106</v>
       </c>
       <c r="Q20" s="10" t="s">
         <v>53</v>
@@ -4576,13 +4664,13 @@
     </row>
     <row r="21" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="14" t="s">
-        <v>113</v>
+        <v>107</v>
       </c>
       <c r="B21" s="14" t="s">
-        <v>114</v>
+        <v>505</v>
       </c>
       <c r="C21" s="15" t="s">
-        <v>496</v>
+        <v>473</v>
       </c>
       <c r="D21" s="12" t="s">
         <v>18</v>
@@ -4591,19 +4679,19 @@
         <v>20</v>
       </c>
       <c r="F21" s="10" t="s">
-        <v>115</v>
+        <v>108</v>
       </c>
       <c r="G21" s="10" t="s">
         <v>33</v>
       </c>
       <c r="H21" s="14" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="I21" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>383</v>
+        <v>360</v>
       </c>
       <c r="K21" s="17" t="s">
         <v>22</v>
@@ -4621,7 +4709,7 @@
         <v>48</v>
       </c>
       <c r="P21" s="14" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="Q21" s="10" t="s">
         <v>53</v>
@@ -4631,13 +4719,13 @@
     </row>
     <row r="22" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14" t="s">
-        <v>118</v>
+        <v>111</v>
       </c>
       <c r="B22" s="14" t="s">
-        <v>119</v>
+        <v>112</v>
       </c>
       <c r="C22" s="15" t="s">
-        <v>495</v>
+        <v>472</v>
       </c>
       <c r="D22" s="12" t="s">
         <v>18</v>
@@ -4646,10 +4734,10 @@
         <v>21</v>
       </c>
       <c r="F22" s="10" t="s">
-        <v>120</v>
+        <v>113</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="H22" s="10" t="s">
         <v>29</v>
@@ -4658,13 +4746,13 @@
         <v>58</v>
       </c>
       <c r="J22" s="37" t="s">
-        <v>384</v>
+        <v>361</v>
       </c>
       <c r="K22" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L22" s="10" t="s">
-        <v>123</v>
+        <v>116</v>
       </c>
       <c r="M22" s="11" t="s">
         <v>22</v>
@@ -4676,7 +4764,7 @@
         <v>48</v>
       </c>
       <c r="P22" s="14" t="s">
-        <v>124</v>
+        <v>117</v>
       </c>
       <c r="Q22" s="10" t="s">
         <v>53</v>
@@ -4686,13 +4774,13 @@
     </row>
     <row r="23" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="14" t="s">
-        <v>125</v>
+        <v>118</v>
       </c>
       <c r="B23" s="14" t="s">
-        <v>126</v>
+        <v>119</v>
       </c>
       <c r="C23" s="15" t="s">
-        <v>127</v>
+        <v>506</v>
       </c>
       <c r="D23" s="12" t="s">
         <v>18</v>
@@ -4701,10 +4789,10 @@
         <v>22</v>
       </c>
       <c r="F23" s="10" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>129</v>
+        <v>121</v>
       </c>
       <c r="H23" s="14" t="s">
         <v>42</v>
@@ -4713,7 +4801,7 @@
         <v>34</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>385</v>
+        <v>362</v>
       </c>
       <c r="K23" s="17" t="s">
         <v>22</v>
@@ -4731,7 +4819,7 @@
         <v>48</v>
       </c>
       <c r="P23" s="14" t="s">
-        <v>130</v>
+        <v>122</v>
       </c>
       <c r="Q23" s="10" t="s">
         <v>53</v>
@@ -4741,13 +4829,13 @@
     </row>
     <row r="24" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="14" t="s">
-        <v>131</v>
+        <v>507</v>
       </c>
       <c r="B24" s="14" t="s">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="C24" s="15" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="D24" s="12" t="s">
         <v>18</v>
@@ -4756,25 +4844,25 @@
         <v>23</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>133</v>
+        <v>124</v>
       </c>
       <c r="G24" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H24" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I24" s="19" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="J24" s="23" t="s">
-        <v>389</v>
+        <v>366</v>
       </c>
       <c r="K24" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L24" s="10" t="s">
-        <v>134</v>
+        <v>125</v>
       </c>
       <c r="M24" s="11" t="s">
         <v>22</v>
@@ -4786,7 +4874,7 @@
         <v>48</v>
       </c>
       <c r="P24" s="14" t="s">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="Q24" s="10" t="s">
         <v>53</v>
@@ -4796,13 +4884,13 @@
     </row>
     <row r="25" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="10" t="s">
-        <v>136</v>
+        <v>127</v>
       </c>
       <c r="B25" s="10" t="s">
-        <v>137</v>
+        <v>128</v>
       </c>
       <c r="C25" s="15" t="s">
-        <v>494</v>
+        <v>471</v>
       </c>
       <c r="D25" s="12" t="s">
         <v>18</v>
@@ -4811,10 +4899,10 @@
         <v>24</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>138</v>
+        <v>129</v>
       </c>
       <c r="G25" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H25" s="14" t="s">
         <v>42</v>
@@ -4823,7 +4911,7 @@
         <v>34</v>
       </c>
       <c r="J25" s="13" t="s">
-        <v>390</v>
+        <v>367</v>
       </c>
       <c r="K25" s="17" t="s">
         <v>22</v>
@@ -4851,13 +4939,13 @@
     </row>
     <row r="26" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="14" t="s">
-        <v>139</v>
+        <v>130</v>
       </c>
       <c r="B26" s="14" t="s">
-        <v>140</v>
+        <v>131</v>
       </c>
       <c r="C26" s="15" t="s">
-        <v>493</v>
+        <v>470</v>
       </c>
       <c r="D26" s="12" t="s">
         <v>18</v>
@@ -4866,37 +4954,37 @@
         <v>25</v>
       </c>
       <c r="F26" s="14" t="s">
-        <v>141</v>
+        <v>132</v>
       </c>
       <c r="G26" s="10" t="s">
-        <v>142</v>
+        <v>133</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="I26" s="10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="J26" s="13" t="s">
-        <v>366</v>
+        <v>343</v>
       </c>
       <c r="K26" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L26" s="14" t="s">
-        <v>143</v>
+        <v>134</v>
       </c>
       <c r="M26" s="11" t="s">
         <v>48</v>
       </c>
       <c r="N26" s="40" t="s">
-        <v>516</v>
+        <v>493</v>
       </c>
       <c r="O26" s="21" t="s">
         <v>48</v>
       </c>
       <c r="P26" s="21" t="s">
-        <v>517</v>
+        <v>494</v>
       </c>
       <c r="Q26" s="10" t="s">
         <v>53</v>
@@ -4906,13 +4994,13 @@
     </row>
     <row r="27" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="10" t="s">
-        <v>144</v>
+        <v>135</v>
       </c>
       <c r="B27" s="14" t="s">
-        <v>145</v>
+        <v>136</v>
       </c>
       <c r="C27" s="15" t="s">
-        <v>492</v>
+        <v>469</v>
       </c>
       <c r="D27" s="12" t="s">
         <v>18</v>
@@ -4921,19 +5009,19 @@
         <v>26</v>
       </c>
       <c r="F27" s="10" t="s">
-        <v>146</v>
+        <v>137</v>
       </c>
       <c r="G27" s="10" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>386</v>
+        <v>363</v>
       </c>
       <c r="I27" s="14" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="J27" s="13" t="s">
-        <v>365</v>
+        <v>342</v>
       </c>
       <c r="K27" s="17" t="s">
         <v>22</v>
@@ -4961,13 +5049,13 @@
     </row>
     <row r="28" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="10" t="s">
-        <v>149</v>
+        <v>140</v>
       </c>
       <c r="B28" s="10" t="s">
-        <v>150</v>
+        <v>141</v>
       </c>
       <c r="C28" s="15" t="s">
-        <v>491</v>
+        <v>468</v>
       </c>
       <c r="D28" s="12" t="s">
         <v>18</v>
@@ -4976,19 +5064,19 @@
         <v>27</v>
       </c>
       <c r="F28" s="10" t="s">
-        <v>151</v>
+        <v>142</v>
       </c>
       <c r="G28" s="10" t="s">
         <v>38</v>
       </c>
       <c r="H28" s="10" t="s">
-        <v>152</v>
+        <v>143</v>
       </c>
       <c r="I28" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J28" s="13" t="s">
-        <v>391</v>
+        <v>368</v>
       </c>
       <c r="K28" s="17" t="s">
         <v>22</v>
@@ -5016,13 +5104,13 @@
     </row>
     <row r="29" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="10" t="s">
-        <v>153</v>
+        <v>144</v>
       </c>
       <c r="B29" s="10" t="s">
-        <v>154</v>
+        <v>508</v>
       </c>
       <c r="C29" s="15" t="s">
-        <v>490</v>
+        <v>467</v>
       </c>
       <c r="D29" s="12" t="s">
         <v>18</v>
@@ -5031,19 +5119,19 @@
         <v>28</v>
       </c>
       <c r="F29" s="10" t="s">
-        <v>155</v>
+        <v>145</v>
       </c>
       <c r="G29" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H29" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I29" s="14" t="s">
-        <v>428</v>
+        <v>405</v>
       </c>
       <c r="J29" s="23" t="s">
-        <v>392</v>
+        <v>369</v>
       </c>
       <c r="K29" s="17" t="s">
         <v>22</v>
@@ -5061,7 +5149,7 @@
         <v>48</v>
       </c>
       <c r="P29" s="14" t="s">
-        <v>156</v>
+        <v>146</v>
       </c>
       <c r="Q29" s="10" t="s">
         <v>53</v>
@@ -5071,13 +5159,13 @@
     </row>
     <row r="30" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
-        <v>157</v>
+        <v>147</v>
       </c>
       <c r="B30" s="10" t="s">
-        <v>158</v>
+        <v>148</v>
       </c>
       <c r="C30" s="15" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="D30" s="12" t="s">
         <v>18</v>
@@ -5086,7 +5174,7 @@
         <v>29</v>
       </c>
       <c r="F30" s="10" t="s">
-        <v>159</v>
+        <v>149</v>
       </c>
       <c r="G30" s="10" t="s">
         <v>46</v>
@@ -5095,10 +5183,10 @@
         <v>42</v>
       </c>
       <c r="I30" s="19" t="s">
-        <v>122</v>
+        <v>115</v>
       </c>
       <c r="J30" s="38" t="s">
-        <v>393</v>
+        <v>370</v>
       </c>
       <c r="K30" s="17" t="s">
         <v>22</v>
@@ -5116,7 +5204,7 @@
         <v>48</v>
       </c>
       <c r="P30" s="14" t="s">
-        <v>160</v>
+        <v>150</v>
       </c>
       <c r="Q30" s="10" t="s">
         <v>53</v>
@@ -5126,13 +5214,13 @@
     </row>
     <row r="31" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="14" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="B31" s="14" t="s">
-        <v>162</v>
+        <v>152</v>
       </c>
       <c r="C31" s="15" t="s">
-        <v>489</v>
+        <v>466</v>
       </c>
       <c r="D31" s="12" t="s">
         <v>18</v>
@@ -5141,7 +5229,7 @@
         <v>30</v>
       </c>
       <c r="F31" s="14" t="s">
-        <v>163</v>
+        <v>153</v>
       </c>
       <c r="G31" s="10" t="s">
         <v>33</v>
@@ -5153,13 +5241,13 @@
         <v>47</v>
       </c>
       <c r="J31" s="23" t="s">
-        <v>394</v>
+        <v>371</v>
       </c>
       <c r="K31" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L31" s="10" t="s">
-        <v>164</v>
+        <v>154</v>
       </c>
       <c r="M31" s="11" t="s">
         <v>22</v>
@@ -5171,27 +5259,27 @@
         <v>48</v>
       </c>
       <c r="P31" s="14" t="s">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="Q31" s="10" t="s">
         <v>53</v>
       </c>
       <c r="R31" s="22" t="s">
-        <v>166</v>
+        <v>499</v>
       </c>
       <c r="S31" s="33" t="s">
-        <v>363</v>
+        <v>340</v>
       </c>
     </row>
     <row r="32" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
-        <v>167</v>
+        <v>156</v>
       </c>
       <c r="B32" s="10" t="s">
-        <v>168</v>
+        <v>157</v>
       </c>
       <c r="C32" s="15" t="s">
-        <v>488</v>
+        <v>465</v>
       </c>
       <c r="D32" s="12" t="s">
         <v>18</v>
@@ -5200,19 +5288,19 @@
         <v>31</v>
       </c>
       <c r="F32" s="10" t="s">
-        <v>169</v>
+        <v>158</v>
       </c>
       <c r="G32" s="10" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="H32" s="14" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="I32" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J32" s="13" t="s">
-        <v>395</v>
+        <v>372</v>
       </c>
       <c r="K32" s="17" t="s">
         <v>22</v>
@@ -5230,7 +5318,7 @@
         <v>48</v>
       </c>
       <c r="P32" s="14" t="s">
-        <v>171</v>
+        <v>160</v>
       </c>
       <c r="Q32" s="10" t="s">
         <v>53</v>
@@ -5240,13 +5328,13 @@
     </row>
     <row r="33" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="10" t="s">
-        <v>172</v>
+        <v>161</v>
       </c>
       <c r="B33" s="10" t="s">
-        <v>173</v>
+        <v>162</v>
       </c>
       <c r="C33" s="15" t="s">
-        <v>174</v>
+        <v>163</v>
       </c>
       <c r="D33" s="12" t="s">
         <v>18</v>
@@ -5255,7 +5343,7 @@
         <v>32</v>
       </c>
       <c r="F33" s="10" t="s">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="G33" s="10" t="s">
         <v>33</v>
@@ -5267,7 +5355,7 @@
         <v>21</v>
       </c>
       <c r="J33" s="13" t="s">
-        <v>396</v>
+        <v>373</v>
       </c>
       <c r="K33" s="17" t="s">
         <v>22</v>
@@ -5285,7 +5373,7 @@
         <v>48</v>
       </c>
       <c r="P33" s="10" t="s">
-        <v>176</v>
+        <v>165</v>
       </c>
       <c r="Q33" s="10" t="s">
         <v>53</v>
@@ -5295,13 +5383,13 @@
     </row>
     <row r="34" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="10" t="s">
-        <v>177</v>
+        <v>166</v>
       </c>
       <c r="B34" s="10" t="s">
-        <v>178</v>
+        <v>167</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>487</v>
+        <v>464</v>
       </c>
       <c r="D34" s="12" t="s">
         <v>18</v>
@@ -5310,19 +5398,19 @@
         <v>33</v>
       </c>
       <c r="F34" s="10" t="s">
-        <v>179</v>
+        <v>168</v>
       </c>
       <c r="G34" s="10" t="s">
-        <v>180</v>
+        <v>169</v>
       </c>
       <c r="H34" s="10" t="s">
-        <v>181</v>
+        <v>497</v>
       </c>
       <c r="I34" s="10" t="s">
         <v>58</v>
       </c>
       <c r="J34" s="23" t="s">
-        <v>397</v>
+        <v>374</v>
       </c>
       <c r="K34" s="17" t="s">
         <v>22</v>
@@ -5350,13 +5438,13 @@
     </row>
     <row r="35" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="14" t="s">
-        <v>182</v>
+        <v>170</v>
       </c>
       <c r="B35" s="14" t="s">
-        <v>183</v>
+        <v>171</v>
       </c>
       <c r="C35" s="15" t="s">
-        <v>486</v>
+        <v>463</v>
       </c>
       <c r="D35" s="12" t="s">
         <v>18</v>
@@ -5365,7 +5453,7 @@
         <v>34</v>
       </c>
       <c r="F35" s="10" t="s">
-        <v>184</v>
+        <v>172</v>
       </c>
       <c r="G35" s="10" t="s">
         <v>46</v>
@@ -5377,13 +5465,13 @@
         <v>58</v>
       </c>
       <c r="J35" s="37" t="s">
-        <v>398</v>
+        <v>375</v>
       </c>
       <c r="K35" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L35" s="10" t="s">
-        <v>185</v>
+        <v>173</v>
       </c>
       <c r="M35" s="11" t="s">
         <v>22</v>
@@ -5395,7 +5483,7 @@
         <v>48</v>
       </c>
       <c r="P35" s="14" t="s">
-        <v>438</v>
+        <v>415</v>
       </c>
       <c r="Q35" s="10" t="s">
         <v>53</v>
@@ -5405,13 +5493,13 @@
     </row>
     <row r="36" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="14" t="s">
-        <v>186</v>
+        <v>174</v>
       </c>
       <c r="B36" s="14" t="s">
-        <v>187</v>
+        <v>175</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>188</v>
+        <v>512</v>
       </c>
       <c r="D36" s="12" t="s">
         <v>18</v>
@@ -5420,10 +5508,10 @@
         <v>35</v>
       </c>
       <c r="F36" s="10" t="s">
-        <v>189</v>
+        <v>176</v>
       </c>
       <c r="G36" s="10" t="s">
-        <v>190</v>
+        <v>177</v>
       </c>
       <c r="H36" s="14" t="s">
         <v>29</v>
@@ -5432,7 +5520,7 @@
         <v>21</v>
       </c>
       <c r="J36" s="24" t="s">
-        <v>399</v>
+        <v>376</v>
       </c>
       <c r="K36" s="17" t="s">
         <v>22</v>
@@ -5450,7 +5538,7 @@
         <v>48</v>
       </c>
       <c r="P36" s="14" t="s">
-        <v>191</v>
+        <v>178</v>
       </c>
       <c r="Q36" s="10" t="s">
         <v>53</v>
@@ -5460,13 +5548,13 @@
     </row>
     <row r="37" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="14" t="s">
-        <v>192</v>
+        <v>509</v>
       </c>
       <c r="B37" s="10" t="s">
-        <v>193</v>
+        <v>179</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>194</v>
+        <v>511</v>
       </c>
       <c r="D37" s="12" t="s">
         <v>18</v>
@@ -5475,10 +5563,10 @@
         <v>36</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>195</v>
+        <v>180</v>
       </c>
       <c r="G37" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H37" s="14" t="s">
         <v>29</v>
@@ -5487,7 +5575,7 @@
         <v>21</v>
       </c>
       <c r="J37" s="25" t="s">
-        <v>400</v>
+        <v>377</v>
       </c>
       <c r="K37" s="17" t="s">
         <v>22</v>
@@ -5505,7 +5593,7 @@
         <v>48</v>
       </c>
       <c r="P37" s="14" t="s">
-        <v>439</v>
+        <v>416</v>
       </c>
       <c r="Q37" s="10" t="s">
         <v>53</v>
@@ -5515,13 +5603,13 @@
     </row>
     <row r="38" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="10" t="s">
-        <v>196</v>
+        <v>181</v>
       </c>
       <c r="B38" s="10" t="s">
-        <v>197</v>
+        <v>182</v>
       </c>
       <c r="C38" s="15" t="s">
-        <v>485</v>
+        <v>462</v>
       </c>
       <c r="D38" s="12" t="s">
         <v>18</v>
@@ -5530,7 +5618,7 @@
         <v>37</v>
       </c>
       <c r="F38" s="10" t="s">
-        <v>198</v>
+        <v>183</v>
       </c>
       <c r="G38" s="10" t="s">
         <v>46</v>
@@ -5542,7 +5630,7 @@
         <v>58</v>
       </c>
       <c r="J38" s="23" t="s">
-        <v>401</v>
+        <v>378</v>
       </c>
       <c r="K38" s="17" t="s">
         <v>22</v>
@@ -5570,13 +5658,13 @@
     </row>
     <row r="39" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="14" t="s">
-        <v>199</v>
+        <v>184</v>
       </c>
       <c r="B39" s="14" t="s">
-        <v>200</v>
+        <v>185</v>
       </c>
       <c r="C39" s="15" t="s">
-        <v>484</v>
+        <v>461</v>
       </c>
       <c r="D39" s="12" t="s">
         <v>18</v>
@@ -5585,7 +5673,7 @@
         <v>38</v>
       </c>
       <c r="F39" s="10" t="s">
-        <v>201</v>
+        <v>186</v>
       </c>
       <c r="G39" s="10" t="s">
         <v>33</v>
@@ -5597,13 +5685,13 @@
         <v>58</v>
       </c>
       <c r="J39" s="37" t="s">
-        <v>398</v>
+        <v>375</v>
       </c>
       <c r="K39" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L39" s="10" t="s">
-        <v>202</v>
+        <v>187</v>
       </c>
       <c r="M39" s="11" t="s">
         <v>22</v>
@@ -5615,7 +5703,7 @@
         <v>48</v>
       </c>
       <c r="P39" s="14" t="s">
-        <v>440</v>
+        <v>417</v>
       </c>
       <c r="Q39" s="10" t="s">
         <v>53</v>
@@ -5624,14 +5712,14 @@
       <c r="S39" s="12"/>
     </row>
     <row r="40" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A40" s="14" t="s">
-        <v>203</v>
+      <c r="A40" s="10" t="s">
+        <v>510</v>
       </c>
       <c r="B40" s="10" t="s">
-        <v>204</v>
+        <v>188</v>
       </c>
       <c r="C40" s="39" t="s">
-        <v>483</v>
+        <v>460</v>
       </c>
       <c r="D40" s="12" t="s">
         <v>18</v>
@@ -5640,19 +5728,19 @@
         <v>39</v>
       </c>
       <c r="F40" s="10" t="s">
-        <v>205</v>
+        <v>189</v>
       </c>
       <c r="G40" s="14" t="s">
-        <v>206</v>
+        <v>190</v>
       </c>
       <c r="H40" s="14" t="s">
-        <v>207</v>
+        <v>191</v>
       </c>
       <c r="I40" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J40" s="13" t="s">
-        <v>402</v>
+        <v>379</v>
       </c>
       <c r="K40" s="17" t="s">
         <v>22</v>
@@ -5679,14 +5767,14 @@
       <c r="S40" s="12"/>
     </row>
     <row r="41" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A41" s="14" t="s">
-        <v>208</v>
+      <c r="A41" s="10" t="s">
+        <v>513</v>
       </c>
       <c r="B41" s="10" t="s">
-        <v>209</v>
+        <v>192</v>
       </c>
       <c r="C41" s="15" t="s">
-        <v>210</v>
+        <v>193</v>
       </c>
       <c r="D41" s="12" t="s">
         <v>18</v>
@@ -5695,19 +5783,19 @@
         <v>40</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>211</v>
+        <v>194</v>
       </c>
       <c r="G41" s="21" t="s">
-        <v>212</v>
+        <v>195</v>
       </c>
       <c r="H41" s="14" t="s">
         <v>29</v>
       </c>
       <c r="I41" s="10" t="s">
-        <v>431</v>
+        <v>408</v>
       </c>
       <c r="J41" s="13" t="s">
-        <v>403</v>
+        <v>380</v>
       </c>
       <c r="K41" s="17" t="s">
         <v>22</v>
@@ -5719,13 +5807,13 @@
         <v>48</v>
       </c>
       <c r="N41" s="40" t="s">
-        <v>213</v>
+        <v>196</v>
       </c>
       <c r="O41" s="18" t="s">
         <v>48</v>
       </c>
       <c r="P41" s="21" t="s">
-        <v>518</v>
+        <v>495</v>
       </c>
       <c r="Q41" s="10" t="s">
         <v>53</v>
@@ -5735,13 +5823,13 @@
     </row>
     <row r="42" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="10" t="s">
-        <v>214</v>
+        <v>197</v>
       </c>
       <c r="B42" s="10" t="s">
-        <v>215</v>
+        <v>198</v>
       </c>
       <c r="C42" s="17" t="s">
-        <v>216</v>
+        <v>199</v>
       </c>
       <c r="D42" s="12" t="s">
         <v>18</v>
@@ -5750,10 +5838,10 @@
         <v>41</v>
       </c>
       <c r="F42" s="10" t="s">
-        <v>217</v>
+        <v>200</v>
       </c>
       <c r="G42" s="10" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H42" s="14" t="s">
         <v>29</v>
@@ -5762,7 +5850,7 @@
         <v>21</v>
       </c>
       <c r="J42" s="13" t="s">
-        <v>404</v>
+        <v>381</v>
       </c>
       <c r="K42" s="17" t="s">
         <v>22</v>
@@ -5780,7 +5868,7 @@
         <v>48</v>
       </c>
       <c r="P42" s="14" t="s">
-        <v>218</v>
+        <v>201</v>
       </c>
       <c r="Q42" s="10" t="s">
         <v>53</v>
@@ -5790,13 +5878,13 @@
     </row>
     <row r="43" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="10" t="s">
-        <v>219</v>
+        <v>202</v>
       </c>
       <c r="B43" s="10" t="s">
-        <v>220</v>
+        <v>203</v>
       </c>
       <c r="C43" s="15" t="s">
-        <v>482</v>
+        <v>459</v>
       </c>
       <c r="D43" s="12" t="s">
         <v>18</v>
@@ -5805,10 +5893,10 @@
         <v>42</v>
       </c>
       <c r="F43" s="10" t="s">
-        <v>221</v>
+        <v>204</v>
       </c>
       <c r="G43" s="10" t="s">
-        <v>222</v>
+        <v>205</v>
       </c>
       <c r="H43" s="14" t="s">
         <v>29</v>
@@ -5817,7 +5905,7 @@
         <v>34</v>
       </c>
       <c r="J43" s="13" t="s">
-        <v>402</v>
+        <v>379</v>
       </c>
       <c r="K43" s="17" t="s">
         <v>22</v>
@@ -5845,13 +5933,13 @@
     </row>
     <row r="44" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="10" t="s">
-        <v>223</v>
+        <v>206</v>
       </c>
       <c r="B44" s="10" t="s">
-        <v>224</v>
+        <v>207</v>
       </c>
       <c r="C44" s="15" t="s">
-        <v>481</v>
+        <v>458</v>
       </c>
       <c r="D44" s="12" t="s">
         <v>18</v>
@@ -5860,7 +5948,7 @@
         <v>43</v>
       </c>
       <c r="F44" s="10" t="s">
-        <v>225</v>
+        <v>208</v>
       </c>
       <c r="G44" s="10" t="s">
         <v>38</v>
@@ -5872,7 +5960,7 @@
         <v>21</v>
       </c>
       <c r="J44" s="37" t="s">
-        <v>405</v>
+        <v>382</v>
       </c>
       <c r="K44" s="17" t="s">
         <v>22</v>
@@ -5900,13 +5988,13 @@
     </row>
     <row r="45" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="14" t="s">
-        <v>226</v>
+        <v>209</v>
       </c>
       <c r="B45" s="14" t="s">
-        <v>227</v>
+        <v>210</v>
       </c>
       <c r="C45" s="15" t="s">
-        <v>228</v>
+        <v>211</v>
       </c>
       <c r="D45" s="12" t="s">
         <v>18</v>
@@ -5915,7 +6003,7 @@
         <v>44</v>
       </c>
       <c r="F45" s="10" t="s">
-        <v>229</v>
+        <v>212</v>
       </c>
       <c r="G45" s="10" t="s">
         <v>46</v>
@@ -5927,13 +6015,13 @@
         <v>34</v>
       </c>
       <c r="J45" s="23" t="s">
-        <v>406</v>
+        <v>383</v>
       </c>
       <c r="K45" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L45" s="10" t="s">
-        <v>230</v>
+        <v>213</v>
       </c>
       <c r="M45" s="11" t="s">
         <v>22</v>
@@ -5945,7 +6033,7 @@
         <v>48</v>
       </c>
       <c r="P45" s="14" t="s">
-        <v>231</v>
+        <v>214</v>
       </c>
       <c r="Q45" s="10" t="s">
         <v>53</v>
@@ -5955,13 +6043,13 @@
     </row>
     <row r="46" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="14" t="s">
-        <v>232</v>
+        <v>215</v>
       </c>
       <c r="B46" s="14" t="s">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="C46" s="15" t="s">
-        <v>480</v>
+        <v>457</v>
       </c>
       <c r="D46" s="12" t="s">
         <v>18</v>
@@ -5970,7 +6058,7 @@
         <v>45</v>
       </c>
       <c r="F46" s="10" t="s">
-        <v>234</v>
+        <v>217</v>
       </c>
       <c r="G46" s="10" t="s">
         <v>46</v>
@@ -5982,13 +6070,13 @@
         <v>47</v>
       </c>
       <c r="J46" s="12" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="K46" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>235</v>
+        <v>218</v>
       </c>
       <c r="M46" s="11" t="s">
         <v>22</v>
@@ -6000,7 +6088,7 @@
         <v>48</v>
       </c>
       <c r="P46" s="14" t="s">
-        <v>441</v>
+        <v>418</v>
       </c>
       <c r="Q46" s="10" t="s">
         <v>53</v>
@@ -6010,13 +6098,13 @@
     </row>
     <row r="47" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="10" t="s">
-        <v>236</v>
+        <v>219</v>
       </c>
       <c r="B47" s="14" t="s">
-        <v>237</v>
+        <v>220</v>
       </c>
       <c r="C47" s="15" t="s">
-        <v>479</v>
+        <v>456</v>
       </c>
       <c r="D47" s="12" t="s">
         <v>18</v>
@@ -6025,19 +6113,19 @@
         <v>46</v>
       </c>
       <c r="F47" s="10" t="s">
-        <v>238</v>
+        <v>221</v>
       </c>
       <c r="G47" s="10" t="s">
-        <v>239</v>
+        <v>222</v>
       </c>
       <c r="H47" s="10" t="s">
-        <v>408</v>
+        <v>385</v>
       </c>
       <c r="I47" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J47" s="16" t="s">
-        <v>409</v>
+        <v>386</v>
       </c>
       <c r="K47" s="17" t="s">
         <v>22</v>
@@ -6055,7 +6143,7 @@
         <v>48</v>
       </c>
       <c r="P47" s="14" t="s">
-        <v>442</v>
+        <v>419</v>
       </c>
       <c r="Q47" s="10" t="s">
         <v>53</v>
@@ -6065,13 +6153,13 @@
     </row>
     <row r="48" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="10" t="s">
-        <v>240</v>
+        <v>223</v>
       </c>
       <c r="B48" s="10" t="s">
-        <v>241</v>
+        <v>224</v>
       </c>
       <c r="C48" s="15" t="s">
-        <v>478</v>
+        <v>455</v>
       </c>
       <c r="D48" s="12" t="s">
         <v>18</v>
@@ -6080,10 +6168,10 @@
         <v>47</v>
       </c>
       <c r="F48" s="10" t="s">
-        <v>242</v>
+        <v>225</v>
       </c>
       <c r="G48" s="10" t="s">
-        <v>243</v>
+        <v>226</v>
       </c>
       <c r="H48" s="10" t="s">
         <v>29</v>
@@ -6092,7 +6180,7 @@
         <v>21</v>
       </c>
       <c r="J48" s="13" t="s">
-        <v>410</v>
+        <v>387</v>
       </c>
       <c r="K48" s="17" t="s">
         <v>22</v>
@@ -6120,13 +6208,13 @@
     </row>
     <row r="49" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="10" t="s">
-        <v>244</v>
+        <v>227</v>
       </c>
       <c r="B49" s="10" t="s">
-        <v>245</v>
+        <v>228</v>
       </c>
       <c r="C49" s="15" t="s">
-        <v>477</v>
+        <v>454</v>
       </c>
       <c r="D49" s="12" t="s">
         <v>18</v>
@@ -6135,10 +6223,10 @@
         <v>48</v>
       </c>
       <c r="F49" s="10" t="s">
-        <v>246</v>
+        <v>229</v>
       </c>
       <c r="G49" s="10" t="s">
-        <v>247</v>
+        <v>230</v>
       </c>
       <c r="H49" s="10" t="s">
         <v>29</v>
@@ -6147,7 +6235,7 @@
         <v>21</v>
       </c>
       <c r="J49" s="13" t="s">
-        <v>411</v>
+        <v>388</v>
       </c>
       <c r="K49" s="17" t="s">
         <v>22</v>
@@ -6175,13 +6263,13 @@
     </row>
     <row r="50" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="10" t="s">
-        <v>248</v>
+        <v>231</v>
       </c>
       <c r="B50" s="10" t="s">
-        <v>249</v>
+        <v>232</v>
       </c>
       <c r="C50" s="15" t="s">
-        <v>476</v>
+        <v>453</v>
       </c>
       <c r="D50" s="12" t="s">
         <v>18</v>
@@ -6190,10 +6278,10 @@
         <v>49</v>
       </c>
       <c r="F50" s="10" t="s">
-        <v>250</v>
+        <v>233</v>
       </c>
       <c r="G50" s="10" t="s">
-        <v>251</v>
+        <v>234</v>
       </c>
       <c r="H50" s="10" t="s">
         <v>29</v>
@@ -6202,7 +6290,7 @@
         <v>21</v>
       </c>
       <c r="J50" s="13" t="s">
-        <v>412</v>
+        <v>389</v>
       </c>
       <c r="K50" s="17" t="s">
         <v>22</v>
@@ -6217,10 +6305,10 @@
         <v>23</v>
       </c>
       <c r="O50" s="10" t="s">
-        <v>252</v>
+        <v>235</v>
       </c>
       <c r="P50" s="14" t="s">
-        <v>443</v>
+        <v>420</v>
       </c>
       <c r="Q50" s="10" t="s">
         <v>53</v>
@@ -6230,13 +6318,13 @@
     </row>
     <row r="51" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="10" t="s">
-        <v>253</v>
+        <v>236</v>
       </c>
       <c r="B51" s="10" t="s">
-        <v>254</v>
+        <v>237</v>
       </c>
       <c r="C51" s="15" t="s">
-        <v>475</v>
+        <v>452</v>
       </c>
       <c r="D51" s="12" t="s">
         <v>18</v>
@@ -6245,19 +6333,19 @@
         <v>50</v>
       </c>
       <c r="F51" s="10" t="s">
-        <v>255</v>
+        <v>238</v>
       </c>
       <c r="G51" s="18" t="s">
-        <v>256</v>
+        <v>239</v>
       </c>
       <c r="H51" s="10" t="s">
         <v>29</v>
       </c>
       <c r="I51" s="10" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="J51" s="13" t="s">
-        <v>367</v>
+        <v>344</v>
       </c>
       <c r="K51" s="17" t="s">
         <v>22</v>
@@ -6269,13 +6357,13 @@
         <v>48</v>
       </c>
       <c r="N51" s="20" t="s">
-        <v>257</v>
+        <v>240</v>
       </c>
       <c r="O51" s="18" t="s">
         <v>48</v>
       </c>
       <c r="P51" s="21" t="s">
-        <v>519</v>
+        <v>496</v>
       </c>
       <c r="Q51" s="10" t="s">
         <v>53</v>
@@ -6285,13 +6373,13 @@
     </row>
     <row r="52" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="14" t="s">
-        <v>258</v>
+        <v>241</v>
       </c>
       <c r="B52" s="14" t="s">
-        <v>259</v>
+        <v>242</v>
       </c>
       <c r="C52" s="15" t="s">
-        <v>474</v>
+        <v>451</v>
       </c>
       <c r="D52" s="12" t="s">
         <v>18</v>
@@ -6300,25 +6388,25 @@
         <v>51</v>
       </c>
       <c r="F52" s="10" t="s">
-        <v>260</v>
+        <v>243</v>
       </c>
       <c r="G52" s="18" t="s">
-        <v>261</v>
+        <v>244</v>
       </c>
       <c r="H52" s="10" t="s">
-        <v>262</v>
+        <v>245</v>
       </c>
       <c r="I52" s="10" t="s">
-        <v>263</v>
+        <v>246</v>
       </c>
       <c r="J52" s="23" t="s">
-        <v>413</v>
+        <v>390</v>
       </c>
       <c r="K52" s="17" t="s">
         <v>48</v>
       </c>
       <c r="L52" s="10" t="s">
-        <v>264</v>
+        <v>247</v>
       </c>
       <c r="M52" s="40" t="s">
         <v>22</v>
@@ -6340,13 +6428,13 @@
     </row>
     <row r="53" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="10" t="s">
-        <v>265</v>
+        <v>248</v>
       </c>
       <c r="B53" s="10" t="s">
-        <v>266</v>
+        <v>249</v>
       </c>
       <c r="C53" s="15" t="s">
-        <v>473</v>
+        <v>450</v>
       </c>
       <c r="D53" s="12" t="s">
         <v>18</v>
@@ -6355,19 +6443,19 @@
         <v>52</v>
       </c>
       <c r="F53" s="10" t="s">
-        <v>267</v>
+        <v>250</v>
       </c>
       <c r="G53" s="10" t="s">
-        <v>170</v>
+        <v>159</v>
       </c>
       <c r="H53" s="10" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="I53" s="10" t="s">
         <v>21</v>
       </c>
       <c r="J53" s="13" t="s">
-        <v>372</v>
+        <v>349</v>
       </c>
       <c r="K53" s="26" t="s">
         <v>22</v>
@@ -6395,13 +6483,13 @@
     </row>
     <row r="54" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="12" t="s">
-        <v>268</v>
+        <v>514</v>
       </c>
       <c r="B54" s="12" t="s">
-        <v>269</v>
+        <v>251</v>
       </c>
       <c r="C54" s="15" t="s">
-        <v>472</v>
+        <v>449</v>
       </c>
       <c r="D54" s="12" t="s">
         <v>18</v>
@@ -6410,7 +6498,7 @@
         <v>53</v>
       </c>
       <c r="F54" s="12" t="s">
-        <v>270</v>
+        <v>252</v>
       </c>
       <c r="G54" s="12" t="s">
         <v>46</v>
@@ -6422,13 +6510,13 @@
         <v>47</v>
       </c>
       <c r="J54" s="12" t="s">
-        <v>414</v>
+        <v>391</v>
       </c>
       <c r="K54" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L54" s="12" t="s">
-        <v>271</v>
+        <v>253</v>
       </c>
       <c r="M54" s="11" t="s">
         <v>22</v>
@@ -6440,23 +6528,23 @@
         <v>48</v>
       </c>
       <c r="P54" s="12" t="s">
-        <v>444</v>
+        <v>421</v>
       </c>
       <c r="Q54" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R54" s="12"/>
       <c r="S54" s="12"/>
     </row>
     <row r="55" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="12" t="s">
-        <v>273</v>
+        <v>255</v>
       </c>
       <c r="B55" s="12" t="s">
-        <v>274</v>
+        <v>256</v>
       </c>
       <c r="C55" s="12" t="s">
-        <v>471</v>
+        <v>448</v>
       </c>
       <c r="D55" s="12" t="s">
         <v>18</v>
@@ -6465,19 +6553,19 @@
         <v>54</v>
       </c>
       <c r="F55" s="12" t="s">
-        <v>275</v>
+        <v>257</v>
       </c>
       <c r="G55" s="12" t="s">
-        <v>276</v>
+        <v>258</v>
       </c>
       <c r="H55" s="12" t="s">
-        <v>387</v>
+        <v>364</v>
       </c>
       <c r="I55" s="12" t="s">
         <v>21</v>
       </c>
       <c r="J55" s="12" t="s">
-        <v>415</v>
+        <v>392</v>
       </c>
       <c r="K55" s="12" t="s">
         <v>22</v>
@@ -6498,20 +6586,20 @@
         <v>23</v>
       </c>
       <c r="Q55" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R55" s="12"/>
       <c r="S55" s="12"/>
     </row>
     <row r="56" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="12" t="s">
-        <v>277</v>
+        <v>259</v>
       </c>
       <c r="B56" s="12" t="s">
-        <v>278</v>
+        <v>260</v>
       </c>
       <c r="C56" s="12" t="s">
-        <v>470</v>
+        <v>447</v>
       </c>
       <c r="D56" s="12" t="s">
         <v>18</v>
@@ -6520,10 +6608,10 @@
         <v>55</v>
       </c>
       <c r="F56" s="12" t="s">
-        <v>279</v>
+        <v>261</v>
       </c>
       <c r="G56" s="12" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="H56" s="12" t="s">
         <v>29</v>
@@ -6532,13 +6620,13 @@
         <v>21</v>
       </c>
       <c r="J56" s="12" t="s">
-        <v>416</v>
+        <v>393</v>
       </c>
       <c r="K56" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L56" s="12" t="s">
-        <v>280</v>
+        <v>262</v>
       </c>
       <c r="M56" s="12" t="s">
         <v>22</v>
@@ -6550,10 +6638,10 @@
         <v>48</v>
       </c>
       <c r="P56" s="12" t="s">
-        <v>445</v>
+        <v>422</v>
       </c>
       <c r="Q56" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R56" s="12"/>
       <c r="S56" s="12"/>
@@ -6566,7 +6654,7 @@
         <v>51</v>
       </c>
       <c r="C57" s="12" t="s">
-        <v>469</v>
+        <v>446</v>
       </c>
       <c r="D57" s="12" t="s">
         <v>18</v>
@@ -6575,7 +6663,7 @@
         <v>56</v>
       </c>
       <c r="F57" s="12" t="s">
-        <v>281</v>
+        <v>263</v>
       </c>
       <c r="G57" s="12" t="s">
         <v>38</v>
@@ -6587,7 +6675,7 @@
         <v>21</v>
       </c>
       <c r="J57" s="16" t="s">
-        <v>373</v>
+        <v>350</v>
       </c>
       <c r="K57" s="12" t="s">
         <v>22</v>
@@ -6608,20 +6696,20 @@
         <v>23</v>
       </c>
       <c r="Q57" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R57" s="12"/>
       <c r="S57" s="12"/>
     </row>
     <row r="58" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="12" t="s">
-        <v>282</v>
+        <v>264</v>
       </c>
       <c r="B58" s="12" t="s">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="C58" s="12" t="s">
-        <v>468</v>
+        <v>445</v>
       </c>
       <c r="D58" s="12" t="s">
         <v>18</v>
@@ -6630,7 +6718,7 @@
         <v>57</v>
       </c>
       <c r="F58" s="12" t="s">
-        <v>283</v>
+        <v>265</v>
       </c>
       <c r="G58" s="12" t="s">
         <v>46</v>
@@ -6642,13 +6730,13 @@
         <v>47</v>
       </c>
       <c r="J58" s="12" t="s">
-        <v>407</v>
+        <v>384</v>
       </c>
       <c r="K58" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L58" s="12" t="s">
-        <v>284</v>
+        <v>266</v>
       </c>
       <c r="M58" s="12" t="s">
         <v>22</v>
@@ -6660,23 +6748,23 @@
         <v>48</v>
       </c>
       <c r="P58" s="12" t="s">
-        <v>446</v>
+        <v>423</v>
       </c>
       <c r="Q58" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R58" s="12"/>
       <c r="S58" s="12"/>
     </row>
     <row r="59" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="12" t="s">
-        <v>285</v>
+        <v>267</v>
       </c>
       <c r="B59" s="12" t="s">
-        <v>286</v>
+        <v>268</v>
       </c>
       <c r="C59" s="12" t="s">
-        <v>467</v>
+        <v>444</v>
       </c>
       <c r="D59" s="12" t="s">
         <v>18</v>
@@ -6685,7 +6773,7 @@
         <v>58</v>
       </c>
       <c r="F59" s="12" t="s">
-        <v>287</v>
+        <v>269</v>
       </c>
       <c r="G59" s="12" t="s">
         <v>33</v>
@@ -6697,13 +6785,13 @@
         <v>47</v>
       </c>
       <c r="J59" s="12" t="s">
-        <v>417</v>
+        <v>394</v>
       </c>
       <c r="K59" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L59" s="12" t="s">
-        <v>288</v>
+        <v>270</v>
       </c>
       <c r="M59" s="12" t="s">
         <v>22</v>
@@ -6715,23 +6803,23 @@
         <v>48</v>
       </c>
       <c r="P59" s="12" t="s">
-        <v>289</v>
+        <v>271</v>
       </c>
       <c r="Q59" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R59" s="12"/>
       <c r="S59" s="12"/>
     </row>
     <row r="60" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="12" t="s">
-        <v>290</v>
+        <v>515</v>
       </c>
       <c r="B60" s="12" t="s">
-        <v>291</v>
+        <v>272</v>
       </c>
       <c r="C60" s="12" t="s">
-        <v>466</v>
+        <v>443</v>
       </c>
       <c r="D60" s="12" t="s">
         <v>18</v>
@@ -6740,25 +6828,25 @@
         <v>59</v>
       </c>
       <c r="F60" s="12" t="s">
-        <v>292</v>
+        <v>273</v>
       </c>
       <c r="G60" s="12" t="s">
-        <v>121</v>
+        <v>114</v>
       </c>
       <c r="H60" s="12" t="s">
         <v>29</v>
       </c>
       <c r="I60" s="12" t="s">
-        <v>293</v>
+        <v>274</v>
       </c>
       <c r="J60" s="23" t="s">
-        <v>418</v>
+        <v>395</v>
       </c>
       <c r="K60" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L60" s="12" t="s">
-        <v>294</v>
+        <v>275</v>
       </c>
       <c r="M60" s="12" t="s">
         <v>22</v>
@@ -6770,23 +6858,23 @@
         <v>48</v>
       </c>
       <c r="P60" s="12" t="s">
-        <v>295</v>
+        <v>276</v>
       </c>
       <c r="Q60" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R60" s="12"/>
       <c r="S60" s="12"/>
     </row>
     <row r="61" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="12" t="s">
-        <v>296</v>
+        <v>277</v>
       </c>
       <c r="B61" s="12" t="s">
-        <v>297</v>
+        <v>278</v>
       </c>
       <c r="C61" s="12" t="s">
-        <v>465</v>
+        <v>442</v>
       </c>
       <c r="D61" s="12" t="s">
         <v>18</v>
@@ -6795,7 +6883,7 @@
         <v>60</v>
       </c>
       <c r="F61" s="12" t="s">
-        <v>298</v>
+        <v>279</v>
       </c>
       <c r="G61" s="12" t="s">
         <v>38</v>
@@ -6807,7 +6895,7 @@
         <v>21</v>
       </c>
       <c r="J61" s="12" t="s">
-        <v>372</v>
+        <v>349</v>
       </c>
       <c r="K61" s="12" t="s">
         <v>22</v>
@@ -6828,20 +6916,20 @@
         <v>23</v>
       </c>
       <c r="Q61" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R61" s="12"/>
       <c r="S61" s="12"/>
     </row>
     <row r="62" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="12" t="s">
-        <v>299</v>
+        <v>516</v>
       </c>
       <c r="B62" s="12" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="C62" s="12" t="s">
-        <v>464</v>
+        <v>441</v>
       </c>
       <c r="D62" s="12" t="s">
         <v>18</v>
@@ -6850,7 +6938,7 @@
         <v>61</v>
       </c>
       <c r="F62" s="12" t="s">
-        <v>301</v>
+        <v>282</v>
       </c>
       <c r="G62" s="12" t="s">
         <v>57</v>
@@ -6862,13 +6950,13 @@
         <v>47</v>
       </c>
       <c r="J62" s="12" t="s">
-        <v>419</v>
+        <v>396</v>
       </c>
       <c r="K62" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L62" s="12" t="s">
-        <v>302</v>
+        <v>283</v>
       </c>
       <c r="M62" s="12" t="s">
         <v>22</v>
@@ -6880,23 +6968,23 @@
         <v>48</v>
       </c>
       <c r="P62" s="12" t="s">
-        <v>447</v>
+        <v>424</v>
       </c>
       <c r="Q62" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R62" s="12"/>
       <c r="S62" s="12"/>
     </row>
     <row r="63" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="12" t="s">
-        <v>303</v>
+        <v>284</v>
       </c>
       <c r="B63" s="12" t="s">
-        <v>304</v>
+        <v>285</v>
       </c>
       <c r="C63" s="12" t="s">
-        <v>463</v>
+        <v>440</v>
       </c>
       <c r="D63" s="12" t="s">
         <v>18</v>
@@ -6905,7 +6993,7 @@
         <v>62</v>
       </c>
       <c r="F63" s="12" t="s">
-        <v>305</v>
+        <v>286</v>
       </c>
       <c r="G63" s="12" t="s">
         <v>57</v>
@@ -6917,7 +7005,7 @@
         <v>34</v>
       </c>
       <c r="J63" s="12" t="s">
-        <v>420</v>
+        <v>397</v>
       </c>
       <c r="K63" s="12" t="s">
         <v>22</v>
@@ -6938,20 +7026,20 @@
         <v>23</v>
       </c>
       <c r="Q63" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R63" s="12"/>
       <c r="S63" s="12"/>
     </row>
     <row r="64" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="12" t="s">
-        <v>306</v>
+        <v>517</v>
       </c>
       <c r="B64" s="12" t="s">
-        <v>307</v>
+        <v>287</v>
       </c>
       <c r="C64" s="12" t="s">
-        <v>462</v>
+        <v>439</v>
       </c>
       <c r="D64" s="12" t="s">
         <v>18</v>
@@ -6960,10 +7048,10 @@
         <v>63</v>
       </c>
       <c r="F64" s="12" t="s">
-        <v>308</v>
+        <v>288</v>
       </c>
       <c r="G64" s="12" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="H64" s="12" t="s">
         <v>42</v>
@@ -6972,7 +7060,7 @@
         <v>21</v>
       </c>
       <c r="J64" s="12" t="s">
-        <v>421</v>
+        <v>398</v>
       </c>
       <c r="K64" s="12" t="s">
         <v>22</v>
@@ -6990,23 +7078,23 @@
         <v>48</v>
       </c>
       <c r="P64" s="12" t="s">
-        <v>448</v>
+        <v>425</v>
       </c>
       <c r="Q64" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R64" s="12"/>
       <c r="S64" s="12"/>
     </row>
     <row r="65" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="12" t="s">
-        <v>309</v>
+        <v>518</v>
       </c>
       <c r="B65" s="12" t="s">
-        <v>310</v>
+        <v>289</v>
       </c>
       <c r="C65" s="12" t="s">
-        <v>461</v>
+        <v>438</v>
       </c>
       <c r="D65" s="12" t="s">
         <v>18</v>
@@ -7015,7 +7103,7 @@
         <v>64</v>
       </c>
       <c r="F65" s="12" t="s">
-        <v>311</v>
+        <v>290</v>
       </c>
       <c r="G65" s="12" t="s">
         <v>46</v>
@@ -7027,13 +7115,13 @@
         <v>34</v>
       </c>
       <c r="J65" s="12" t="s">
-        <v>422</v>
+        <v>399</v>
       </c>
       <c r="K65" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L65" s="12" t="s">
-        <v>299</v>
+        <v>280</v>
       </c>
       <c r="M65" s="12" t="s">
         <v>22</v>
@@ -7045,23 +7133,23 @@
         <v>48</v>
       </c>
       <c r="P65" s="12" t="s">
-        <v>449</v>
+        <v>426</v>
       </c>
       <c r="Q65" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R65" s="12"/>
       <c r="S65" s="12"/>
     </row>
     <row r="66" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="12" t="s">
-        <v>312</v>
+        <v>519</v>
       </c>
       <c r="B66" s="12" t="s">
-        <v>313</v>
+        <v>291</v>
       </c>
       <c r="C66" s="12" t="s">
-        <v>460</v>
+        <v>437</v>
       </c>
       <c r="D66" s="12" t="s">
         <v>18</v>
@@ -7070,7 +7158,7 @@
         <v>65</v>
       </c>
       <c r="F66" s="12" t="s">
-        <v>314</v>
+        <v>292</v>
       </c>
       <c r="G66" s="12" t="s">
         <v>33</v>
@@ -7082,7 +7170,7 @@
         <v>34</v>
       </c>
       <c r="J66" s="12" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="K66" s="12" t="s">
         <v>22</v>
@@ -7103,20 +7191,20 @@
         <v>23</v>
       </c>
       <c r="Q66" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R66" s="12"/>
       <c r="S66" s="12"/>
     </row>
     <row r="67" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="12" t="s">
-        <v>315</v>
+        <v>293</v>
       </c>
       <c r="B67" s="12" t="s">
-        <v>316</v>
+        <v>294</v>
       </c>
       <c r="C67" s="12" t="s">
-        <v>459</v>
+        <v>436</v>
       </c>
       <c r="D67" s="12" t="s">
         <v>18</v>
@@ -7125,10 +7213,10 @@
         <v>66</v>
       </c>
       <c r="F67" s="12" t="s">
-        <v>317</v>
+        <v>295</v>
       </c>
       <c r="G67" s="12" t="s">
-        <v>318</v>
+        <v>296</v>
       </c>
       <c r="H67" s="12" t="s">
         <v>29</v>
@@ -7137,7 +7225,7 @@
         <v>21</v>
       </c>
       <c r="J67" s="12" t="s">
-        <v>423</v>
+        <v>400</v>
       </c>
       <c r="K67" s="12" t="s">
         <v>22</v>
@@ -7158,20 +7246,20 @@
         <v>23</v>
       </c>
       <c r="Q67" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R67" s="12"/>
       <c r="S67" s="12"/>
     </row>
     <row r="68" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="12" t="s">
-        <v>319</v>
+        <v>297</v>
       </c>
       <c r="B68" s="12" t="s">
-        <v>320</v>
+        <v>298</v>
       </c>
       <c r="C68" s="12" t="s">
-        <v>458</v>
+        <v>435</v>
       </c>
       <c r="D68" s="12" t="s">
         <v>18</v>
@@ -7180,7 +7268,7 @@
         <v>67</v>
       </c>
       <c r="F68" s="12" t="s">
-        <v>321</v>
+        <v>299</v>
       </c>
       <c r="G68" s="12" t="s">
         <v>46</v>
@@ -7192,13 +7280,13 @@
         <v>47</v>
       </c>
       <c r="J68" s="12" t="s">
-        <v>424</v>
+        <v>401</v>
       </c>
       <c r="K68" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L68" s="12" t="s">
-        <v>322</v>
+        <v>300</v>
       </c>
       <c r="M68" s="12" t="s">
         <v>22</v>
@@ -7210,23 +7298,23 @@
         <v>48</v>
       </c>
       <c r="P68" s="12" t="s">
-        <v>450</v>
+        <v>427</v>
       </c>
       <c r="Q68" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R68" s="12"/>
       <c r="S68" s="12"/>
     </row>
     <row r="69" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="12" t="s">
-        <v>299</v>
+        <v>516</v>
       </c>
       <c r="B69" s="12" t="s">
-        <v>300</v>
+        <v>281</v>
       </c>
       <c r="C69" s="12" t="s">
-        <v>457</v>
+        <v>434</v>
       </c>
       <c r="D69" s="12" t="s">
         <v>18</v>
@@ -7235,10 +7323,10 @@
         <v>68</v>
       </c>
       <c r="F69" s="12" t="s">
-        <v>323</v>
+        <v>301</v>
       </c>
       <c r="G69" s="12" t="s">
-        <v>432</v>
+        <v>409</v>
       </c>
       <c r="H69" s="12" t="s">
         <v>29</v>
@@ -7247,13 +7335,13 @@
         <v>47</v>
       </c>
       <c r="J69" s="12" t="s">
-        <v>425</v>
+        <v>402</v>
       </c>
       <c r="K69" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L69" s="12" t="s">
-        <v>324</v>
+        <v>302</v>
       </c>
       <c r="M69" s="12" t="s">
         <v>22</v>
@@ -7265,23 +7353,23 @@
         <v>48</v>
       </c>
       <c r="P69" s="12" t="s">
-        <v>451</v>
+        <v>428</v>
       </c>
       <c r="Q69" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R69" s="12"/>
       <c r="S69" s="12"/>
     </row>
     <row r="70" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="12" t="s">
-        <v>325</v>
+        <v>303</v>
       </c>
       <c r="B70" s="12" t="s">
-        <v>326</v>
+        <v>304</v>
       </c>
       <c r="C70" s="12" t="s">
-        <v>456</v>
+        <v>433</v>
       </c>
       <c r="D70" s="12" t="s">
         <v>18</v>
@@ -7290,19 +7378,19 @@
         <v>69</v>
       </c>
       <c r="F70" s="12" t="s">
-        <v>327</v>
+        <v>305</v>
       </c>
       <c r="G70" s="12" t="s">
-        <v>328</v>
+        <v>306</v>
       </c>
       <c r="H70" s="12" t="s">
-        <v>388</v>
+        <v>365</v>
       </c>
       <c r="I70" s="12" t="s">
         <v>34</v>
       </c>
       <c r="J70" s="12" t="s">
-        <v>426</v>
+        <v>403</v>
       </c>
       <c r="K70" s="12" t="s">
         <v>22</v>
@@ -7323,20 +7411,20 @@
         <v>23</v>
       </c>
       <c r="Q70" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R70" s="12"/>
       <c r="S70" s="12"/>
     </row>
     <row r="71" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="12" t="s">
-        <v>329</v>
+        <v>520</v>
       </c>
       <c r="B71" s="12" t="s">
-        <v>330</v>
+        <v>307</v>
       </c>
       <c r="C71" s="12" t="s">
-        <v>455</v>
+        <v>432</v>
       </c>
       <c r="D71" s="12" t="s">
         <v>18</v>
@@ -7345,10 +7433,10 @@
         <v>70</v>
       </c>
       <c r="F71" s="12" t="s">
-        <v>331</v>
+        <v>308</v>
       </c>
       <c r="G71" s="12" t="s">
-        <v>332</v>
+        <v>309</v>
       </c>
       <c r="H71" s="12" t="s">
         <v>29</v>
@@ -7357,13 +7445,13 @@
         <v>47</v>
       </c>
       <c r="J71" s="12" t="s">
-        <v>427</v>
+        <v>404</v>
       </c>
       <c r="K71" s="12" t="s">
         <v>48</v>
       </c>
       <c r="L71" s="12" t="s">
-        <v>333</v>
+        <v>310</v>
       </c>
       <c r="M71" s="12" t="s">
         <v>22</v>
@@ -7375,23 +7463,23 @@
         <v>48</v>
       </c>
       <c r="P71" s="12" t="s">
-        <v>452</v>
+        <v>429</v>
       </c>
       <c r="Q71" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R71" s="12"/>
       <c r="S71" s="12"/>
     </row>
     <row r="72" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="12" t="s">
-        <v>334</v>
+        <v>311</v>
       </c>
       <c r="B72" s="12" t="s">
-        <v>335</v>
+        <v>312</v>
       </c>
       <c r="C72" s="12" t="s">
-        <v>454</v>
+        <v>431</v>
       </c>
       <c r="D72" s="12" t="s">
         <v>18</v>
@@ -7400,19 +7488,19 @@
         <v>71</v>
       </c>
       <c r="F72" s="12" t="s">
-        <v>336</v>
+        <v>313</v>
       </c>
       <c r="G72" s="12" t="s">
-        <v>337</v>
+        <v>314</v>
       </c>
       <c r="H72" s="12" t="s">
-        <v>338</v>
+        <v>315</v>
       </c>
       <c r="I72" s="12" t="s">
-        <v>148</v>
+        <v>139</v>
       </c>
       <c r="J72" s="12" t="s">
-        <v>339</v>
+        <v>316</v>
       </c>
       <c r="K72" s="12" t="s">
         <v>22</v>
@@ -7433,20 +7521,20 @@
         <v>23</v>
       </c>
       <c r="Q72" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R72" s="12"/>
       <c r="S72" s="12"/>
     </row>
     <row r="73" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="12" t="s">
-        <v>340</v>
+        <v>317</v>
       </c>
       <c r="B73" s="12" t="s">
-        <v>341</v>
+        <v>318</v>
       </c>
       <c r="C73" s="12" t="s">
-        <v>453</v>
+        <v>430</v>
       </c>
       <c r="D73" s="12" t="s">
         <v>18</v>
@@ -7455,19 +7543,19 @@
         <v>72</v>
       </c>
       <c r="F73" s="12" t="s">
-        <v>342</v>
+        <v>319</v>
       </c>
       <c r="G73" s="12" t="s">
-        <v>343</v>
+        <v>320</v>
       </c>
       <c r="H73" s="12" t="s">
-        <v>344</v>
+        <v>321</v>
       </c>
       <c r="I73" s="12" t="s">
         <v>58</v>
       </c>
       <c r="J73" s="12" t="s">
-        <v>430</v>
+        <v>407</v>
       </c>
       <c r="K73" s="12" t="s">
         <v>22</v>
@@ -7488,7 +7576,7 @@
         <v>23</v>
       </c>
       <c r="Q73" s="12" t="s">
-        <v>272</v>
+        <v>254</v>
       </c>
       <c r="R73" s="12"/>
       <c r="S73" s="12"/>
@@ -8565,66 +8653,66 @@
   <sheetData>
     <row r="1" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="27" t="s">
-        <v>345</v>
+        <v>322</v>
       </c>
       <c r="B1" s="27" t="s">
-        <v>346</v>
+        <v>323</v>
       </c>
       <c r="C1" s="27" t="s">
-        <v>347</v>
+        <v>324</v>
       </c>
       <c r="D1" s="27" t="s">
-        <v>348</v>
+        <v>325</v>
       </c>
       <c r="E1" s="27" t="s">
-        <v>349</v>
+        <v>326</v>
       </c>
       <c r="F1" s="27" t="s">
-        <v>350</v>
+        <v>327</v>
       </c>
       <c r="G1" s="27" t="s">
-        <v>351</v>
+        <v>328</v>
       </c>
       <c r="H1" s="28" t="s">
-        <v>352</v>
+        <v>329</v>
       </c>
       <c r="I1" s="28" t="s">
-        <v>353</v>
+        <v>330</v>
       </c>
       <c r="J1" s="29" t="s">
-        <v>354</v>
+        <v>331</v>
       </c>
     </row>
     <row r="2" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="30" t="s">
-        <v>355</v>
+        <v>332</v>
       </c>
       <c r="B2" s="30" t="s">
-        <v>356</v>
+        <v>333</v>
       </c>
       <c r="C2" s="30" t="s">
-        <v>357</v>
+        <v>334</v>
       </c>
       <c r="D2" s="30" t="s">
-        <v>358</v>
+        <v>335</v>
       </c>
       <c r="E2" s="30" t="s">
         <v>29</v>
       </c>
       <c r="F2" s="30" t="s">
-        <v>359</v>
+        <v>336</v>
       </c>
       <c r="G2" s="31" t="s">
-        <v>360</v>
+        <v>337</v>
       </c>
       <c r="H2" s="35" t="s">
         <v>23</v>
       </c>
       <c r="I2" s="32" t="s">
-        <v>361</v>
+        <v>338</v>
       </c>
       <c r="J2" s="31" t="s">
-        <v>362</v>
+        <v>339</v>
       </c>
     </row>
     <row r="3" spans="1:10" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>

</xml_diff>